<commit_message>
SBT: normalize currency in matches-only workbook; add review CSV; docs/gitignore updated
</commit_message>
<xml_diff>
--- a/Estelita/Processed/Unificado SBT nov dez 23 e jan fev mar 24__matches_only_with_refs.xlsx
+++ b/Estelita/Processed/Unificado SBT nov dez 23 e jan fev mar 24__matches_only_with_refs.xlsx
@@ -558,7 +558,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -630,7 +630,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -702,7 +702,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -846,7 +846,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>599,79</t>
+          <t>R$ 599,79</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -918,7 +918,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -990,7 +990,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>199,93</t>
+          <t>R$ 199,93</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1062,7 +1062,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1134,7 +1134,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1270,7 +1270,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1342,7 +1342,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
@@ -1482,7 +1482,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -1550,7 +1550,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -1618,7 +1618,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -1686,7 +1686,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -1826,7 +1826,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>533,09</t>
+          <t>R$ 533,09</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>266,62</t>
+          <t>R$ 266,62</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>299,89</t>
+          <t>R$ 299,89</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2042,7 +2042,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>99,96</t>
+          <t>R$ 99,96</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -2330,7 +2330,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -2470,7 +2470,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -2538,7 +2538,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -2750,7 +2750,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -2822,7 +2822,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>538,53</t>
+          <t>R$ 538,53</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>261,19</t>
+          <t>R$ 261,19</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>79,97</t>
+          <t>R$ 79,97</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>1519,46</t>
+          <t>R$ 1.519,46</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
@@ -3326,7 +3326,7 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
@@ -3466,7 +3466,7 @@
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>1199,57</t>
+          <t>R$ 1.199,57</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
@@ -3538,7 +3538,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
@@ -3682,7 +3682,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
@@ -3754,7 +3754,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>373,70</t>
+          <t>R$ 373,70</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
@@ -3826,7 +3826,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>373,70</t>
+          <t>R$ 373,70</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -3966,7 +3966,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
@@ -4038,7 +4038,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
@@ -4110,7 +4110,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
@@ -4182,7 +4182,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
@@ -4254,7 +4254,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>159,94</t>
+          <t>R$ 159,94</t>
         </is>
       </c>
       <c r="M54" t="inlineStr">
@@ -4326,7 +4326,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>639,77</t>
+          <t>R$ 639,77</t>
         </is>
       </c>
       <c r="M55" t="inlineStr">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M56" t="inlineStr">
@@ -4470,7 +4470,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>199,93</t>
+          <t>R$ 199,93</t>
         </is>
       </c>
       <c r="M57" t="inlineStr">
@@ -4542,7 +4542,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>199,93</t>
+          <t>R$ 199,93</t>
         </is>
       </c>
       <c r="M58" t="inlineStr">
@@ -4614,7 +4614,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M59" t="inlineStr">
@@ -4686,7 +4686,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M60" t="inlineStr">
@@ -4758,7 +4758,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M61" t="inlineStr">
@@ -4830,7 +4830,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M62" t="inlineStr">
@@ -4898,7 +4898,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M63" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M64" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>599,78</t>
+          <t>R$ 599,78</t>
         </is>
       </c>
       <c r="M65" t="inlineStr">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>199,93</t>
+          <t>R$ 199,93</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M67" t="inlineStr">
@@ -5258,7 +5258,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M68" t="inlineStr">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M69" t="inlineStr">
@@ -5402,7 +5402,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M70" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M71" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>533,09</t>
+          <t>R$ 533,09</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -5614,7 +5614,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>1066,34</t>
+          <t>R$ 1.066,34</t>
         </is>
       </c>
       <c r="M73" t="inlineStr">
@@ -5686,7 +5686,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>299,89</t>
+          <t>R$ 299,89</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -5758,7 +5758,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M75" t="inlineStr">
@@ -5830,7 +5830,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>99,96</t>
+          <t>R$ 99,96</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -5902,7 +5902,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>1199,57</t>
+          <t>R$ 1.199,57</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -5974,7 +5974,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -6046,7 +6046,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -6118,7 +6118,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>1599,43</t>
+          <t>R$ 1.599,43</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -6190,7 +6190,7 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
@@ -6262,7 +6262,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>799,71</t>
+          <t>R$ 799,71</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -6402,7 +6402,7 @@
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>299,89</t>
+          <t>R$ 299,89</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -6474,7 +6474,7 @@
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M85" t="inlineStr">
@@ -6546,7 +6546,7 @@
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>99,96</t>
+          <t>R$ 99,96</t>
         </is>
       </c>
       <c r="M86" t="inlineStr">
@@ -6618,7 +6618,7 @@
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>533,09</t>
+          <t>R$ 533,09</t>
         </is>
       </c>
       <c r="M87" t="inlineStr">
@@ -6690,7 +6690,7 @@
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>266,62</t>
+          <t>R$ 266,62</t>
         </is>
       </c>
       <c r="M88" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>799,72</t>
+          <t>R$ 799,72</t>
         </is>
       </c>
       <c r="M89" t="inlineStr">
@@ -6830,7 +6830,7 @@
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M90" t="inlineStr">
@@ -6898,7 +6898,7 @@
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>399,86</t>
+          <t>R$ 399,86</t>
         </is>
       </c>
       <c r="M91" t="inlineStr">
@@ -6964,8 +6964,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L92" t="n">
-        <v>390.96</v>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -7034,8 +7036,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L93" t="n">
-        <v>1673.31</v>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -7104,8 +7108,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L94" t="n">
-        <v>836.65</v>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
@@ -7174,8 +7180,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L95" t="n">
-        <v>1673.31</v>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -7244,8 +7252,10 @@
           <t>33.33%</t>
         </is>
       </c>
-      <c r="L96" t="n">
-        <v>557.71</v>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>R$ 55.771,00</t>
+        </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
@@ -7314,8 +7324,10 @@
           <t>66.67%</t>
         </is>
       </c>
-      <c r="L97" t="n">
-        <v>1115.6</v>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>R$ 11.156,00</t>
+        </is>
       </c>
       <c r="M97" t="inlineStr">
         <is>
@@ -7384,8 +7396,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L98" t="n">
-        <v>1673.31</v>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M98" t="inlineStr">
         <is>
@@ -7454,8 +7468,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L99" t="n">
-        <v>1673.31</v>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -7524,8 +7540,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L100" t="n">
-        <v>836.65</v>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
@@ -7594,8 +7612,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L101" t="n">
-        <v>836.65</v>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
@@ -7660,8 +7680,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L102" t="n">
-        <v>418.32</v>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>R$ 41.832,00</t>
+        </is>
       </c>
       <c r="M102" t="inlineStr">
         <is>
@@ -7730,8 +7752,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L103" t="n">
-        <v>418.32</v>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>R$ 41.832,00</t>
+        </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -7800,8 +7824,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L104" t="n">
-        <v>836.65</v>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M104" t="inlineStr">
         <is>
@@ -7866,8 +7892,10 @@
           <t>25.00%</t>
         </is>
       </c>
-      <c r="L105" t="n">
-        <v>209.16</v>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>R$ 20.916,00</t>
+        </is>
       </c>
       <c r="M105" t="inlineStr">
         <is>
@@ -7936,8 +7964,10 @@
           <t>75.00%</t>
         </is>
       </c>
-      <c r="L106" t="n">
-        <v>627.49</v>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>R$ 62.749,00</t>
+        </is>
       </c>
       <c r="M106" t="inlineStr">
         <is>
@@ -8006,8 +8036,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L107" t="n">
-        <v>1673.31</v>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M107" t="inlineStr">
         <is>
@@ -8076,8 +8108,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L108" t="n">
-        <v>836.65</v>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M108" t="inlineStr">
         <is>
@@ -8146,8 +8180,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L109" t="n">
-        <v>836.65</v>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M109" t="inlineStr">
         <is>
@@ -8216,8 +8252,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L110" t="n">
-        <v>836.65</v>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -8286,8 +8324,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L111" t="n">
-        <v>836.65</v>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -8356,8 +8396,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L112" t="n">
-        <v>836.65</v>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -8422,8 +8464,10 @@
           <t>16.66%</t>
         </is>
       </c>
-      <c r="L113" t="n">
-        <v>139.39</v>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>R$ 13.939,00</t>
+        </is>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -8492,8 +8536,10 @@
           <t>83.34%</t>
         </is>
       </c>
-      <c r="L114" t="n">
-        <v>697.26</v>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>R$ 69.726,00</t>
+        </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>
@@ -8562,8 +8608,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L115" t="n">
-        <v>1673.31</v>
+      <c r="L115" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M115" t="inlineStr">
         <is>
@@ -8632,8 +8680,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L116" t="n">
-        <v>836.66</v>
+      <c r="L116" t="inlineStr">
+        <is>
+          <t>R$ 83.666,00</t>
+        </is>
       </c>
       <c r="M116" t="inlineStr">
         <is>
@@ -8702,8 +8752,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L117" t="n">
-        <v>836.66</v>
+      <c r="L117" t="inlineStr">
+        <is>
+          <t>R$ 83.666,00</t>
+        </is>
       </c>
       <c r="M117" t="inlineStr">
         <is>
@@ -8772,8 +8824,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L118" t="n">
-        <v>836.65</v>
+      <c r="L118" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M118" t="inlineStr">
         <is>
@@ -8842,8 +8896,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L119" t="n">
-        <v>836.65</v>
+      <c r="L119" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M119" t="inlineStr">
         <is>
@@ -8908,8 +8964,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L120" t="n">
-        <v>1673.31</v>
+      <c r="L120" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M120" t="inlineStr">
         <is>
@@ -8978,8 +9036,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L121" t="n">
-        <v>836.66</v>
+      <c r="L121" t="inlineStr">
+        <is>
+          <t>R$ 83.666,00</t>
+        </is>
       </c>
       <c r="M121" t="inlineStr">
         <is>
@@ -9048,8 +9108,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L122" t="n">
-        <v>836.66</v>
+      <c r="L122" t="inlineStr">
+        <is>
+          <t>R$ 83.666,00</t>
+        </is>
       </c>
       <c r="M122" t="inlineStr">
         <is>
@@ -9118,8 +9180,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L123" t="n">
-        <v>836.65</v>
+      <c r="L123" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M123" t="inlineStr">
         <is>
@@ -9188,8 +9252,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L124" t="n">
-        <v>418.32</v>
+      <c r="L124" t="inlineStr">
+        <is>
+          <t>R$ 41.832,00</t>
+        </is>
       </c>
       <c r="M124" t="inlineStr">
         <is>
@@ -9258,8 +9324,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L125" t="n">
-        <v>418.32</v>
+      <c r="L125" t="inlineStr">
+        <is>
+          <t>R$ 41.832,00</t>
+        </is>
       </c>
       <c r="M125" t="inlineStr">
         <is>
@@ -9330,7 +9398,7 @@
       </c>
       <c r="L126" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M126" t="inlineStr">
@@ -9398,7 +9466,7 @@
       </c>
       <c r="L127" t="inlineStr">
         <is>
-          <t>390,96</t>
+          <t>R$ 390,96</t>
         </is>
       </c>
       <c r="M127" t="inlineStr">
@@ -9470,7 +9538,7 @@
       </c>
       <c r="L128" t="inlineStr">
         <is>
-          <t>260,73</t>
+          <t>R$ 260,73</t>
         </is>
       </c>
       <c r="M128" t="inlineStr">
@@ -9542,7 +9610,7 @@
       </c>
       <c r="L129" t="inlineStr">
         <is>
-          <t>130,23</t>
+          <t>R$ 130,23</t>
         </is>
       </c>
       <c r="M129" t="inlineStr">
@@ -9614,7 +9682,7 @@
       </c>
       <c r="L130" t="inlineStr">
         <is>
-          <t>390,96</t>
+          <t>R$ 390,96</t>
         </is>
       </c>
       <c r="M130" t="inlineStr">
@@ -9682,7 +9750,7 @@
       </c>
       <c r="L131" t="inlineStr">
         <is>
-          <t>390,96</t>
+          <t>R$ 390,96</t>
         </is>
       </c>
       <c r="M131" t="inlineStr">
@@ -9754,7 +9822,7 @@
       </c>
       <c r="L132" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M132" t="inlineStr">
@@ -9826,7 +9894,7 @@
       </c>
       <c r="L133" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M133" t="inlineStr">
@@ -9898,7 +9966,7 @@
       </c>
       <c r="L134" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M134" t="inlineStr">
@@ -9970,7 +10038,7 @@
       </c>
       <c r="L135" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M135" t="inlineStr">
@@ -10042,7 +10110,7 @@
       </c>
       <c r="L136" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M136" t="inlineStr">
@@ -10114,7 +10182,7 @@
       </c>
       <c r="L137" t="inlineStr">
         <is>
-          <t>1673,31</t>
+          <t>R$ 1.673,31</t>
         </is>
       </c>
       <c r="M137" t="inlineStr">
@@ -10186,7 +10254,7 @@
       </c>
       <c r="L138" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M138" t="inlineStr">
@@ -10258,7 +10326,7 @@
       </c>
       <c r="L139" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M139" t="inlineStr">
@@ -10330,7 +10398,7 @@
       </c>
       <c r="L140" t="inlineStr">
         <is>
-          <t>1673,31</t>
+          <t>R$ 1.673,31</t>
         </is>
       </c>
       <c r="M140" t="inlineStr">
@@ -10402,7 +10470,7 @@
       </c>
       <c r="L141" t="inlineStr">
         <is>
-          <t>334,66</t>
+          <t>R$ 334,66</t>
         </is>
       </c>
       <c r="M141" t="inlineStr">
@@ -10474,7 +10542,7 @@
       </c>
       <c r="L142" t="inlineStr">
         <is>
-          <t>334,66</t>
+          <t>R$ 334,66</t>
         </is>
       </c>
       <c r="M142" t="inlineStr">
@@ -10546,7 +10614,7 @@
       </c>
       <c r="L143" t="inlineStr">
         <is>
-          <t>669,32</t>
+          <t>R$ 669,32</t>
         </is>
       </c>
       <c r="M143" t="inlineStr">
@@ -10618,7 +10686,7 @@
       </c>
       <c r="L144" t="inlineStr">
         <is>
-          <t>334,66</t>
+          <t>R$ 334,66</t>
         </is>
       </c>
       <c r="M144" t="inlineStr">
@@ -10690,7 +10758,7 @@
       </c>
       <c r="L145" t="inlineStr">
         <is>
-          <t>1673,31</t>
+          <t>R$ 1.673,31</t>
         </is>
       </c>
       <c r="M145" t="inlineStr">
@@ -10762,7 +10830,7 @@
       </c>
       <c r="L146" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M146" t="inlineStr">
@@ -10830,7 +10898,7 @@
       </c>
       <c r="L147" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M147" t="inlineStr">
@@ -10898,7 +10966,7 @@
       </c>
       <c r="L148" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M148" t="inlineStr">
@@ -10966,7 +11034,7 @@
       </c>
       <c r="L149" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M149" t="inlineStr">
@@ -11038,7 +11106,7 @@
       </c>
       <c r="L150" t="inlineStr">
         <is>
-          <t>585,66</t>
+          <t>R$ 585,66</t>
         </is>
       </c>
       <c r="M150" t="inlineStr">
@@ -11110,7 +11178,7 @@
       </c>
       <c r="L151" t="inlineStr">
         <is>
-          <t>251,00</t>
+          <t>R$ 251,00</t>
         </is>
       </c>
       <c r="M151" t="inlineStr">
@@ -11182,7 +11250,7 @@
       </c>
       <c r="L152" t="inlineStr">
         <is>
-          <t>585,66</t>
+          <t>R$ 585,66</t>
         </is>
       </c>
       <c r="M152" t="inlineStr">
@@ -11254,7 +11322,7 @@
       </c>
       <c r="L153" t="inlineStr">
         <is>
-          <t>251,00</t>
+          <t>R$ 251,00</t>
         </is>
       </c>
       <c r="M153" t="inlineStr">
@@ -11326,7 +11394,7 @@
       </c>
       <c r="L154" t="inlineStr">
         <is>
-          <t>92,03</t>
+          <t>R$ 92,03</t>
         </is>
       </c>
       <c r="M154" t="inlineStr">
@@ -11398,7 +11466,7 @@
       </c>
       <c r="L155" t="inlineStr">
         <is>
-          <t>744,62</t>
+          <t>R$ 744,62</t>
         </is>
       </c>
       <c r="M155" t="inlineStr">
@@ -11470,7 +11538,7 @@
       </c>
       <c r="L156" t="inlineStr">
         <is>
-          <t>836,65</t>
+          <t>R$ 836,65</t>
         </is>
       </c>
       <c r="M156" t="inlineStr">
@@ -11542,7 +11610,7 @@
       </c>
       <c r="L157" t="inlineStr">
         <is>
-          <t>278,77</t>
+          <t>R$ 278,77</t>
         </is>
       </c>
       <c r="M157" t="inlineStr">
@@ -11614,7 +11682,7 @@
       </c>
       <c r="L158" t="inlineStr">
         <is>
-          <t>1394,54</t>
+          <t>R$ 1.394,54</t>
         </is>
       </c>
       <c r="M158" t="inlineStr">
@@ -11682,8 +11750,10 @@
           <t>33.33%</t>
         </is>
       </c>
-      <c r="L159" t="n">
-        <v>130.31</v>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>R$ 13.031,00</t>
+        </is>
       </c>
       <c r="M159" t="inlineStr">
         <is>
@@ -11750,8 +11820,10 @@
           <t>66.67%</t>
         </is>
       </c>
-      <c r="L160" t="n">
-        <v>260.65</v>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>R$ 26.065,00</t>
+        </is>
       </c>
       <c r="M160" t="inlineStr">
         <is>
@@ -11818,8 +11890,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L161" t="n">
-        <v>1673.31</v>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M161" t="inlineStr">
         <is>
@@ -11886,8 +11960,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L162" t="n">
-        <v>390.96</v>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M162" t="inlineStr">
         <is>
@@ -11950,8 +12026,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L163" t="n">
-        <v>390.96</v>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M163" t="inlineStr">
         <is>
@@ -12018,8 +12096,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L164" t="n">
-        <v>390.96</v>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
@@ -12086,8 +12166,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L165" t="n">
-        <v>195.48</v>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>R$ 19.548,00</t>
+        </is>
       </c>
       <c r="M165" t="inlineStr">
         <is>
@@ -12150,8 +12232,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L166" t="n">
-        <v>195.48</v>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>R$ 19.548,00</t>
+        </is>
       </c>
       <c r="M166" t="inlineStr">
         <is>
@@ -12214,8 +12298,10 @@
           <t>5.00%</t>
         </is>
       </c>
-      <c r="L167" t="n">
-        <v>39.1</v>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>R$ 391,00</t>
+        </is>
       </c>
       <c r="M167" t="inlineStr">
         <is>
@@ -12282,8 +12368,10 @@
           <t>95.00%</t>
         </is>
       </c>
-      <c r="L168" t="n">
-        <v>742.8200000000001</v>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>R$ 74.282,00</t>
+        </is>
       </c>
       <c r="M168" t="inlineStr">
         <is>
@@ -12350,8 +12438,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L169" t="n">
-        <v>781.92</v>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>R$ 78.192,00</t>
+        </is>
       </c>
       <c r="M169" t="inlineStr">
         <is>
@@ -12418,8 +12508,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L170" t="n">
-        <v>836.65</v>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>R$ 83.665,00</t>
+        </is>
       </c>
       <c r="M170" t="inlineStr">
         <is>
@@ -12486,8 +12578,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L171" t="n">
-        <v>781.92</v>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>R$ 78.192,00</t>
+        </is>
       </c>
       <c r="M171" t="inlineStr">
         <is>
@@ -12554,8 +12648,10 @@
           <t>50.00%</t>
         </is>
       </c>
-      <c r="L172" t="n">
-        <v>390.96</v>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M172" t="inlineStr">
         <is>
@@ -12618,8 +12714,10 @@
           <t>25.00%</t>
         </is>
       </c>
-      <c r="L173" t="n">
-        <v>195.48</v>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>R$ 19.548,00</t>
+        </is>
       </c>
       <c r="M173" t="inlineStr">
         <is>
@@ -12682,8 +12780,10 @@
           <t>25.00%</t>
         </is>
       </c>
-      <c r="L174" t="n">
-        <v>195.48</v>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>R$ 19.548,00</t>
+        </is>
       </c>
       <c r="M174" t="inlineStr">
         <is>
@@ -12746,8 +12846,10 @@
           <t>5.82%</t>
         </is>
       </c>
-      <c r="L175" t="n">
-        <v>22.75</v>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>R$ 2.275,00</t>
+        </is>
       </c>
       <c r="M175" t="inlineStr">
         <is>
@@ -12814,8 +12916,10 @@
           <t>5.84%</t>
         </is>
       </c>
-      <c r="L176" t="n">
-        <v>22.83</v>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>R$ 2.283,00</t>
+        </is>
       </c>
       <c r="M176" t="inlineStr">
         <is>
@@ -12882,8 +12986,10 @@
           <t>88.34%</t>
         </is>
       </c>
-      <c r="L177" t="n">
-        <v>345.37</v>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>R$ 34.537,00</t>
+        </is>
       </c>
       <c r="M177" t="inlineStr">
         <is>
@@ -12950,8 +13056,10 @@
           <t>75.86%</t>
         </is>
       </c>
-      <c r="L178" t="n">
-        <v>296.58</v>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>R$ 29.658,00</t>
+        </is>
       </c>
       <c r="M178" t="inlineStr">
         <is>
@@ -13014,8 +13122,10 @@
           <t>24.14%</t>
         </is>
       </c>
-      <c r="L179" t="n">
-        <v>94.38</v>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>R$ 9.438,00</t>
+        </is>
       </c>
       <c r="M179" t="inlineStr">
         <is>
@@ -13078,8 +13188,10 @@
           <t>75.00%</t>
         </is>
       </c>
-      <c r="L180" t="n">
-        <v>293.22</v>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>R$ 29.322,00</t>
+        </is>
       </c>
       <c r="M180" t="inlineStr">
         <is>
@@ -13146,8 +13258,10 @@
           <t>25.00%</t>
         </is>
       </c>
-      <c r="L181" t="n">
-        <v>97.73999999999999</v>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>R$ 9.774,00</t>
+        </is>
       </c>
       <c r="M181" t="inlineStr">
         <is>
@@ -13214,8 +13328,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L182" t="n">
-        <v>781.92</v>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>R$ 78.192,00</t>
+        </is>
       </c>
       <c r="M182" t="inlineStr">
         <is>
@@ -13282,8 +13398,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L183" t="n">
-        <v>390.96</v>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M183" t="inlineStr">
         <is>
@@ -13350,8 +13468,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L184" t="n">
-        <v>390.96</v>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M184" t="inlineStr">
         <is>
@@ -13414,8 +13534,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L185" t="n">
-        <v>390.96</v>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M185" t="inlineStr">
         <is>
@@ -13482,8 +13604,10 @@
           <t>33.33%</t>
         </is>
       </c>
-      <c r="L186" t="n">
-        <v>130.31</v>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>R$ 13.031,00</t>
+        </is>
       </c>
       <c r="M186" t="inlineStr">
         <is>
@@ -13550,8 +13674,10 @@
           <t>66.67%</t>
         </is>
       </c>
-      <c r="L187" t="n">
-        <v>260.65</v>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>R$ 26.065,00</t>
+        </is>
       </c>
       <c r="M187" t="inlineStr">
         <is>
@@ -13618,8 +13744,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L188" t="n">
-        <v>1673.31</v>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>R$ 167.331,00</t>
+        </is>
       </c>
       <c r="M188" t="inlineStr">
         <is>
@@ -13686,8 +13814,10 @@
           <t>100.00%</t>
         </is>
       </c>
-      <c r="L189" t="n">
-        <v>390.96</v>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>R$ 39.096,00</t>
+        </is>
       </c>
       <c r="M189" t="inlineStr">
         <is>

</xml_diff>